<commit_message>
feat: Implement Excel and JSON loaders for portfolio and tax data
- Added ExcelSchemaLoader for cleaning and validating Excel sheets.
- Introduced PortfolioInputSource with ExcelPortfolioLoader and JSONPortfolioLoader for loading portfolio data.
- Created TaxTable class for loading tax-related data from Excel.
- Enhanced export utilities for logging and debugging.
- Updated withdrawal simulation logic to incorporate Roth conversion and RMD suppression.
- Refactored portfolio preparation and validation processes.
- Improved Streamlit integration for portfolio data input.
- Adjusted import paths for consistency across modules.
</commit_message>
<xml_diff>
--- a/data/import/tax_table.xlsx
+++ b/data/import/tax_table.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="9300" yWindow="75" windowWidth="28080" windowHeight="11025" firstSheet="1" activeTab="7"/>
+    <workbookView xWindow="9300" yWindow="75" windowWidth="28080" windowHeight="11025" firstSheet="1" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="T_AMT" sheetId="16" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="96">
   <si>
     <t>Single</t>
   </si>
@@ -269,6 +269,54 @@
   </si>
   <si>
     <t>H_PCT</t>
+  </si>
+  <si>
+    <t>QD</t>
+  </si>
+  <si>
+    <t>QD %</t>
+  </si>
+  <si>
+    <t>OD%</t>
+  </si>
+  <si>
+    <t>Interest %</t>
+  </si>
+  <si>
+    <t>LTCG %</t>
+  </si>
+  <si>
+    <t>Taxable Portfolio</t>
+  </si>
+  <si>
+    <t>Yield Type</t>
+  </si>
+  <si>
+    <t>Future Target</t>
+  </si>
+  <si>
+    <t>Interest</t>
+  </si>
+  <si>
+    <t>0.3–0.7%</t>
+  </si>
+  <si>
+    <t>0.7–1.2%</t>
+  </si>
+  <si>
+    <t>OD</t>
+  </si>
+  <si>
+    <t>0.1–0.3%</t>
+  </si>
+  <si>
+    <t>LTCG</t>
+  </si>
+  <si>
+    <t>0–0.5%</t>
+  </si>
+  <si>
+    <t>* Tax Efficient allocation for 60/40 Portfolio</t>
   </si>
 </sst>
 </file>
@@ -390,7 +438,7 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -459,6 +507,11 @@
     <xf numFmtId="10" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="10" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Calculation" xfId="4" builtinId="22"/>
@@ -884,15 +937,15 @@
       <c r="F2" s="33">
         <v>0</v>
       </c>
-      <c r="G2" s="26" t="str">
+      <c r="G2" s="38" t="str">
         <f>IF(D2=0,"",(D2/D5-1))</f>
         <v/>
       </c>
-      <c r="H2" s="26" t="str">
+      <c r="H2" s="38" t="str">
         <f t="shared" ref="H2:I4" si="0">IF(E2=0,"",(E2/E5-1))</f>
         <v/>
       </c>
-      <c r="I2" s="26" t="str">
+      <c r="I2" s="38" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
@@ -916,15 +969,15 @@
       <c r="F3" s="33">
         <v>66200</v>
       </c>
-      <c r="G3" s="26">
+      <c r="G3" s="38">
         <f t="shared" ref="G3:G4" si="1">IF(D3=0,"",(D3/D6-1))</f>
         <v>2.2750775594622574E-2</v>
       </c>
-      <c r="H3" s="26">
+      <c r="H3" s="38">
         <f t="shared" si="0"/>
         <v>2.2750775594622574E-2</v>
       </c>
-      <c r="I3" s="26">
+      <c r="I3" s="38">
         <f t="shared" si="0"/>
         <v>2.2393822393822482E-2</v>
       </c>
@@ -948,15 +1001,15 @@
       <c r="F4" s="33">
         <v>579600</v>
       </c>
-      <c r="G4" s="26">
+      <c r="G4" s="38">
         <f t="shared" si="1"/>
         <v>2.2684664416947831E-2</v>
       </c>
-      <c r="H4" s="26">
+      <c r="H4" s="38">
         <f t="shared" si="0"/>
         <v>2.2748104324639584E-2</v>
       </c>
-      <c r="I4" s="26">
+      <c r="I4" s="38">
         <f t="shared" si="0"/>
         <v>2.276336686077296E-2</v>
       </c>
@@ -980,6 +1033,9 @@
       <c r="F5" s="33">
         <v>0</v>
       </c>
+      <c r="G5" s="38"/>
+      <c r="H5" s="38"/>
+      <c r="I5" s="38"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="18">
@@ -1000,6 +1056,9 @@
       <c r="F6" s="33">
         <v>64750</v>
       </c>
+      <c r="G6" s="38"/>
+      <c r="H6" s="38"/>
+      <c r="I6" s="38"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="18">
@@ -1020,6 +1079,9 @@
       <c r="F7" s="33">
         <v>566700</v>
       </c>
+      <c r="G7" s="38"/>
+      <c r="H7" s="38"/>
+      <c r="I7" s="38"/>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="21"/>
@@ -1109,15 +1171,15 @@
         <v>17700</v>
       </c>
       <c r="J2" s="38">
-        <f>IF(E2=-1,"",(E2/E10)-1)</f>
+        <f t="shared" ref="J2:J8" si="0">IF(E2=-1,"",(E2/E10)-1)</f>
         <v>3.98322851153039E-2</v>
       </c>
       <c r="K2" s="38">
-        <f>IF(G2=-1,"",(G2/G10)-1)</f>
+        <f t="shared" ref="K2:K8" si="1">IF(G2=-1,"",(G2/G10)-1)</f>
         <v>3.98322851153039E-2</v>
       </c>
       <c r="L2" s="38">
-        <f>IF(I2=-1,"",(I2/I10)-1)</f>
+        <f t="shared" ref="L2:L8" si="2">IF(I2=-1,"",(I2/I10)-1)</f>
         <v>4.117647058823537E-2</v>
       </c>
     </row>
@@ -1153,15 +1215,15 @@
         <v>67450</v>
       </c>
       <c r="J3" s="38">
-        <f>IF(E3=-1,"",(E3/E11)-1)</f>
+        <f t="shared" si="0"/>
         <v>3.971119133573997E-2</v>
       </c>
       <c r="K3" s="38">
-        <f>IF(G3=-1,"",(G3/G11)-1)</f>
+        <f t="shared" si="1"/>
         <v>3.971119133573997E-2</v>
       </c>
       <c r="L3" s="38">
-        <f>IF(I3=-1,"",(I3/I11)-1)</f>
+        <f t="shared" si="2"/>
         <v>4.0092521202775622E-2</v>
       </c>
     </row>
@@ -1176,36 +1238,36 @@
         <v>0.22</v>
       </c>
       <c r="D4" s="32">
-        <f t="shared" ref="D4:D8" si="0">E3+1</f>
+        <f t="shared" ref="D4:D8" si="3">E3+1</f>
         <v>50401</v>
       </c>
       <c r="E4" s="33">
         <v>105700</v>
       </c>
       <c r="F4" s="32">
-        <f t="shared" ref="F4:F8" si="1">G3+1</f>
+        <f t="shared" ref="F4:F8" si="4">G3+1</f>
         <v>100801</v>
       </c>
       <c r="G4" s="33">
         <v>211400</v>
       </c>
       <c r="H4" s="32">
-        <f t="shared" ref="H4:H8" si="2">I3+1</f>
+        <f t="shared" ref="H4:H8" si="5">I3+1</f>
         <v>67451</v>
       </c>
       <c r="I4" s="33">
         <v>105700</v>
       </c>
       <c r="J4" s="38">
-        <f>IF(E4=-1,"",(E4/E12)-1)</f>
+        <f t="shared" si="0"/>
         <v>2.2738268021286867E-2</v>
       </c>
       <c r="K4" s="38">
-        <f>IF(G4=-1,"",(G4/G12)-1)</f>
+        <f t="shared" si="1"/>
         <v>2.2738268021286867E-2</v>
       </c>
       <c r="L4" s="38">
-        <f>IF(I4=-1,"",(I4/I12)-1)</f>
+        <f t="shared" si="2"/>
         <v>2.2738268021286867E-2</v>
       </c>
     </row>
@@ -1220,36 +1282,36 @@
         <v>0.24</v>
       </c>
       <c r="D5" s="32">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>105701</v>
       </c>
       <c r="E5" s="33">
         <v>201775</v>
       </c>
       <c r="F5" s="32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>211401</v>
       </c>
       <c r="G5" s="33">
         <v>403550</v>
       </c>
       <c r="H5" s="32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>105701</v>
       </c>
       <c r="I5" s="33">
         <v>201750</v>
       </c>
       <c r="J5" s="38">
-        <f>IF(E5=-1,"",(E5/E13)-1)</f>
+        <f t="shared" si="0"/>
         <v>2.2681196147998017E-2</v>
       </c>
       <c r="K5" s="38">
-        <f>IF(G5=-1,"",(G5/G13)-1)</f>
+        <f t="shared" si="1"/>
         <v>2.2681196147998017E-2</v>
       </c>
       <c r="L5" s="38">
-        <f>IF(I5=-1,"",(I5/I13)-1)</f>
+        <f t="shared" si="2"/>
         <v>2.2554485554992398E-2</v>
       </c>
     </row>
@@ -1264,36 +1326,36 @@
         <v>0.32</v>
       </c>
       <c r="D6" s="32">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>201776</v>
       </c>
       <c r="E6" s="33">
         <v>256226</v>
       </c>
       <c r="F6" s="32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>403551</v>
       </c>
       <c r="G6" s="33">
         <v>512450</v>
       </c>
       <c r="H6" s="32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>201751</v>
       </c>
       <c r="I6" s="33">
         <v>256200</v>
       </c>
       <c r="J6" s="38">
-        <f>IF(E6=-1,"",(E6/E14)-1)</f>
+        <f t="shared" si="0"/>
         <v>2.2756211954894745E-2</v>
       </c>
       <c r="K6" s="38">
-        <f>IF(G6=-1,"",(G6/G14)-1)</f>
+        <f t="shared" si="1"/>
         <v>2.2752220337291629E-2</v>
       </c>
       <c r="L6" s="38">
-        <f>IF(I6=-1,"",(I6/I14)-1)</f>
+        <f t="shared" si="2"/>
         <v>2.2754491017964007E-2</v>
       </c>
     </row>
@@ -1308,36 +1370,36 @@
         <v>0.35</v>
       </c>
       <c r="D7" s="32">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>256227</v>
       </c>
       <c r="E7" s="33">
         <v>640600</v>
       </c>
       <c r="F7" s="32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>512451</v>
       </c>
       <c r="G7" s="33">
         <v>768700</v>
       </c>
       <c r="H7" s="32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>256201</v>
       </c>
       <c r="I7" s="33">
         <v>640600</v>
       </c>
       <c r="J7" s="38">
-        <f>IF(E7=-1,"",(E7/E15)-1)</f>
+        <f t="shared" si="0"/>
         <v>2.2750858146403763E-2</v>
       </c>
       <c r="K7" s="38">
-        <f>IF(G7=-1,"",(G7/G15)-1)</f>
+        <f t="shared" si="1"/>
         <v>2.2751463544438577E-2</v>
       </c>
       <c r="L7" s="38">
-        <f>IF(I7=-1,"",(I7/I15)-1)</f>
+        <f t="shared" si="2"/>
         <v>2.2750858146403763E-2</v>
       </c>
     </row>
@@ -1352,36 +1414,36 @@
         <v>0.37</v>
       </c>
       <c r="D8" s="32">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>640601</v>
       </c>
       <c r="E8" s="33">
         <v>-1</v>
       </c>
       <c r="F8" s="32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>768701</v>
       </c>
       <c r="G8" s="33">
         <v>-1</v>
       </c>
       <c r="H8" s="32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>640601</v>
       </c>
       <c r="I8" s="33">
         <v>-1</v>
       </c>
       <c r="J8" s="38" t="str">
-        <f>IF(E8=-1,"",(E8/E16)-1)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="K8" s="38" t="str">
-        <f>IF(G8=-1,"",(G8/G16)-1)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="L8" s="38" t="str">
-        <f>IF(I8=-1,"",(I8/I16)-1)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
@@ -1466,7 +1528,7 @@
         <v>0.22</v>
       </c>
       <c r="D12" s="32">
-        <f t="shared" ref="D12:D16" si="3">E11+1</f>
+        <f t="shared" ref="D12:D16" si="6">E11+1</f>
         <v>48476</v>
       </c>
       <c r="E12" s="33">
@@ -1480,7 +1542,7 @@
         <v>206700</v>
       </c>
       <c r="H12" s="32">
-        <f t="shared" ref="H12:H16" si="4">I11+1</f>
+        <f t="shared" ref="H12:H16" si="7">I11+1</f>
         <v>64851</v>
       </c>
       <c r="I12" s="33">
@@ -1498,21 +1560,21 @@
         <v>0.24</v>
       </c>
       <c r="D13" s="32">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>103351</v>
       </c>
       <c r="E13" s="33">
         <v>197300</v>
       </c>
       <c r="F13" s="32">
-        <f t="shared" ref="F13:F16" si="5">G12+1</f>
+        <f t="shared" ref="F13:F16" si="8">G12+1</f>
         <v>206701</v>
       </c>
       <c r="G13" s="33">
         <v>394600</v>
       </c>
       <c r="H13" s="32">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v>103351</v>
       </c>
       <c r="I13" s="33">
@@ -1530,21 +1592,21 @@
         <v>0.32</v>
       </c>
       <c r="D14" s="32">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>197301</v>
       </c>
       <c r="E14" s="33">
         <v>250525</v>
       </c>
       <c r="F14" s="32">
-        <f t="shared" si="5"/>
+        <f t="shared" si="8"/>
         <v>394601</v>
       </c>
       <c r="G14" s="33">
         <v>501050</v>
       </c>
       <c r="H14" s="32">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v>197301</v>
       </c>
       <c r="I14" s="33">
@@ -1562,21 +1624,21 @@
         <v>0.35</v>
       </c>
       <c r="D15" s="32">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>250526</v>
       </c>
       <c r="E15" s="33">
         <v>626350</v>
       </c>
       <c r="F15" s="32">
-        <f t="shared" si="5"/>
+        <f t="shared" si="8"/>
         <v>501051</v>
       </c>
       <c r="G15" s="33">
         <v>751600</v>
       </c>
       <c r="H15" s="32">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v>250501</v>
       </c>
       <c r="I15" s="33">
@@ -1594,21 +1656,21 @@
         <v>0.37</v>
       </c>
       <c r="D16" s="32">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>626351</v>
       </c>
       <c r="E16" s="33">
         <v>-1</v>
       </c>
       <c r="F16" s="32">
-        <f t="shared" si="5"/>
+        <f t="shared" si="8"/>
         <v>751601</v>
       </c>
       <c r="G16" s="33">
         <v>-1</v>
       </c>
       <c r="H16" s="32">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v>626351</v>
       </c>
       <c r="I16" s="33">
@@ -1689,11 +1751,11 @@
         <v>2.2222222222222143E-2</v>
       </c>
       <c r="G2" s="38">
-        <f>IF(D3="",0,(D2/D3)-1)</f>
+        <f t="shared" ref="G2:H7" si="1">IF(D3="",0,(D2/D3)-1)</f>
         <v>2.2222222222222143E-2</v>
       </c>
       <c r="H2" s="38">
-        <f>IF(E3="",0,(E2/E3)-1)</f>
+        <f t="shared" si="1"/>
         <v>2.2222222222222143E-2</v>
       </c>
       <c r="I2"/>
@@ -1722,11 +1784,11 @@
         <v>7.8767123287671215E-2</v>
       </c>
       <c r="G3" s="38">
-        <f>IF(D4="",0,(D3/D4)-1)</f>
+        <f t="shared" si="1"/>
         <v>7.8767123287671215E-2</v>
       </c>
       <c r="H3" s="38">
-        <f>IF(E4="",0,(E3/E4)-1)</f>
+        <f t="shared" si="1"/>
         <v>7.8767123287671215E-2</v>
       </c>
     </row>
@@ -1751,11 +1813,11 @@
         <v>5.4151624548736566E-2</v>
       </c>
       <c r="G4" s="38">
-        <f>IF(D5="",0,(D4/D5)-1)</f>
+        <f t="shared" si="1"/>
         <v>5.4151624548736566E-2</v>
       </c>
       <c r="H4" s="38">
-        <f>IF(E5="",0,(E4/E5)-1)</f>
+        <f t="shared" si="1"/>
         <v>5.2884615384615419E-2</v>
       </c>
     </row>
@@ -1780,11 +1842,11 @@
         <v>6.9498069498069581E-2</v>
       </c>
       <c r="G5" s="38">
-        <f>IF(D6="",0,(D5/D6)-1)</f>
+        <f t="shared" si="1"/>
         <v>6.9498069498069581E-2</v>
       </c>
       <c r="H5" s="38">
-        <f>IF(E6="",0,(E5/E6)-1)</f>
+        <f t="shared" si="1"/>
         <v>7.2164948453608213E-2</v>
       </c>
     </row>
@@ -1809,11 +1871,11 @@
         <v>3.1872509960159334E-2</v>
       </c>
       <c r="G6" s="38">
-        <f>IF(D7="",0,(D6/D7)-1)</f>
+        <f t="shared" si="1"/>
         <v>3.1872509960159334E-2</v>
       </c>
       <c r="H6" s="38">
-        <f>IF(E7="",0,(E6/E7)-1)</f>
+        <f t="shared" si="1"/>
         <v>3.1914893617021267E-2</v>
       </c>
     </row>
@@ -1838,11 +1900,11 @@
         <v>1.2096774193548487E-2</v>
       </c>
       <c r="G7" s="38">
-        <f>IF(D8="",0,(D7/D8)-1)</f>
+        <f t="shared" si="1"/>
         <v>1.2096774193548487E-2</v>
       </c>
       <c r="H7" s="38">
-        <f>IF(E8="",0,(E7/E8)-1)</f>
+        <f t="shared" si="1"/>
         <v>8.0428954423592547E-3</v>
       </c>
     </row>
@@ -4714,16 +4776,19 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="5" width="11.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13" bestFit="1" customWidth="1"/>
+    <col min="7" max="10" width="9.140625" style="44"/>
+    <col min="11" max="11" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>19</v>
       </c>
@@ -4742,8 +4807,26 @@
       <c r="F1" s="3">
         <v>2026</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" s="43" t="s">
+        <v>83</v>
+      </c>
+      <c r="H1" s="43" t="s">
+        <v>81</v>
+      </c>
+      <c r="I1" s="43" t="s">
+        <v>82</v>
+      </c>
+      <c r="J1" s="43" t="s">
+        <v>84</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>71</v>
       </c>
@@ -4762,8 +4845,30 @@
       <c r="F2" s="6">
         <v>106371</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G2" s="44">
+        <f>$F3/$F12</f>
+        <v>8.0180952380952374E-3</v>
+      </c>
+      <c r="H2" s="44">
+        <f>$F4/$F12</f>
+        <v>7.8680952380952383E-3</v>
+      </c>
+      <c r="I2" s="44">
+        <f>$F5/$F12</f>
+        <v>2.4709999999999999E-2</v>
+      </c>
+      <c r="J2" s="44">
+        <f>$F8/$F12</f>
+        <v>3.1041428571428571E-2</v>
+      </c>
+      <c r="K2" t="s">
+        <v>88</v>
+      </c>
+      <c r="L2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -4782,8 +4887,14 @@
       <c r="F3" s="5">
         <v>16838</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="K3" t="s">
+        <v>80</v>
+      </c>
+      <c r="L3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>13</v>
       </c>
@@ -4802,8 +4913,14 @@
       <c r="F4" s="5">
         <v>16523</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="K4" t="s">
+        <v>91</v>
+      </c>
+      <c r="L4" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>14</v>
       </c>
@@ -4822,8 +4939,14 @@
       <c r="F5" s="5">
         <v>51891</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="K5" t="s">
+        <v>93</v>
+      </c>
+      <c r="L5" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>15</v>
       </c>
@@ -4842,8 +4965,11 @@
       <c r="F6" s="5">
         <v>4714</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="K6" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>73</v>
       </c>
@@ -4863,7 +4989,7 @@
         <v>7227</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>16</v>
       </c>
@@ -4883,7 +5009,7 @@
         <v>65187</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>17</v>
       </c>
@@ -4900,7 +5026,7 @@
         <v>14640</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>18</v>
       </c>
@@ -4923,8 +5049,17 @@
         <v>252228</v>
       </c>
     </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>85</v>
+      </c>
+      <c r="F12" s="42">
+        <v>2100000</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>